<commit_message>
Update readme with latest functionality and ticket
</commit_message>
<xml_diff>
--- a/ticket-tracker.xlsx
+++ b/ticket-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhatt\projects\codex\between-the-lines\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6FB046B-4F23-4666-B090-6C7E5107AB27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E7311B4-13D9-4E79-972D-AD895F2D2769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
   <si>
     <t>Project Ticket Tracker</t>
   </si>
@@ -108,17 +108,29 @@
     <t>Open</t>
   </si>
   <si>
-    <t>Bhatt</t>
-  </si>
-  <si>
     <t>Follow-up after basic login page implementation.</t>
+  </si>
+  <si>
+    <t>FE-002</t>
+  </si>
+  <si>
+    <t>UI enhancements with adornments and basic validation</t>
+  </si>
+  <si>
+    <t>Move from useRef to useState for inputs, disabled submit until fields are filled, basic email validation for email field, password visibility toggle, start input adornments with icons</t>
+  </si>
+  <si>
+    <t>In Prod</t>
+  </si>
+  <si>
+    <t>Vikram Bhat</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -138,6 +150,10 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -188,7 +204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -199,17 +215,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="7">
     <dxf>
       <font>
         <b/>
@@ -233,71 +255,6 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FFD9E1F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF375623"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF5F497A"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFE4DFEC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF843C0C"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF1F4E79"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -528,7 +485,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="438" row="0">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -558,13 +515,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="28.05" customHeight="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
+      <c r="B1" s="5"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -572,7 +529,7 @@
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="1">
@@ -581,7 +538,7 @@
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="1">
@@ -590,7 +547,7 @@
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="1">
@@ -599,7 +556,7 @@
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="1">
@@ -608,7 +565,7 @@
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -625,21 +582,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="16.69921875" customWidth="1"/>
-    <col min="3" max="3" width="46.69921875" customWidth="1"/>
-    <col min="4" max="4" width="63.296875" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="16.69921875" customWidth="1"/>
-    <col min="8" max="8" width="18.296875" customWidth="1"/>
-    <col min="9" max="9" width="46.69921875" customWidth="1"/>
+    <col min="1" max="1" width="15" style="6" customWidth="1"/>
+    <col min="2" max="2" width="16.69921875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="46.69921875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="63.296875" style="6" customWidth="1"/>
+    <col min="5" max="5" width="15" style="6" customWidth="1"/>
+    <col min="6" max="6" width="20" style="6" customWidth="1"/>
+    <col min="7" max="7" width="16.69921875" style="6" customWidth="1"/>
+    <col min="8" max="8" width="18.296875" style="6" customWidth="1"/>
+    <col min="9" max="9" width="46.69921875" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.796875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="24" customHeight="1">
+    <row r="1" spans="1:9">
       <c r="A1" s="2" t="s">
         <v>9</v>
       </c>
@@ -668,7 +626,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="48" customHeight="1">
+    <row r="2" spans="1:9" ht="27.6">
       <c r="A2" s="3" t="s">
         <v>18</v>
       </c>
@@ -685,50 +643,65 @@
         <v>22</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>2</v>
       </c>
       <c r="I2" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="41.4">
+      <c r="A3" s="6" t="s">
         <v>25</v>
       </c>
+      <c r="B3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" s="7">
+        <v>46137</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="F2:F200">
     <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
       <formula>"Open"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F200">
     <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F200">
     <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
       <formula>"Blocked"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F200">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
       <formula>"In Review"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F200">
     <cfRule type="cellIs" dxfId="2" priority="5" operator="equal">
       <formula>"Done"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F200">
     <cfRule type="cellIs" dxfId="1" priority="6" operator="equal">
       <formula>"Staging"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F200">
     <cfRule type="cellIs" dxfId="0" priority="7" operator="equal">
       <formula>"In Prod"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add auth logic with /login endpoint
</commit_message>
<xml_diff>
--- a/ticket-tracker.xlsx
+++ b/ticket-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhatt\projects\codex\between-the-lines\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E7311B4-13D9-4E79-972D-AD895F2D2769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8178975E-67E7-4177-BA6E-03E60D591946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
   <si>
     <t>Project Ticket Tracker</t>
   </si>
@@ -124,6 +124,21 @@
   </si>
   <si>
     <t>Vikram Bhat</t>
+  </si>
+  <si>
+    <t>BE-001</t>
+  </si>
+  <si>
+    <t>Backend</t>
+  </si>
+  <si>
+    <t>Login endpoint wired with JWT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wire in JWT token and controller, service and db layer. Use Postgres and docker for db. </t>
+  </si>
+  <si>
+    <t>Staging</t>
   </si>
 </sst>
 </file>
@@ -204,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -218,14 +233,17 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -515,10 +533,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="28.05" customHeight="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
+      <c r="B1" s="7"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="4" t="s">
@@ -582,19 +600,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="15" style="6" customWidth="1"/>
-    <col min="2" max="2" width="16.69921875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="46.69921875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="63.296875" style="6" customWidth="1"/>
-    <col min="5" max="5" width="15" style="6" customWidth="1"/>
-    <col min="6" max="6" width="20" style="6" customWidth="1"/>
-    <col min="7" max="7" width="16.69921875" style="6" customWidth="1"/>
-    <col min="8" max="8" width="18.296875" style="6" customWidth="1"/>
-    <col min="9" max="9" width="46.69921875" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.796875" style="6"/>
+    <col min="1" max="1" width="15" style="5" customWidth="1"/>
+    <col min="2" max="2" width="16.69921875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="46.69921875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="63.296875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="15" style="5" customWidth="1"/>
+    <col min="6" max="6" width="20" style="5" customWidth="1"/>
+    <col min="7" max="7" width="16.69921875" style="5" customWidth="1"/>
+    <col min="8" max="8" width="18.296875" style="5" customWidth="1"/>
+    <col min="9" max="9" width="46.69921875" style="5" customWidth="1"/>
+    <col min="10" max="16384" width="8.796875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -656,28 +674,54 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="41.4">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>23</v>
+      <c r="F3" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H3" s="7">
+      <c r="H3" s="6">
+        <v>46137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="27.6">
+      <c r="A4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="8">
         <v>46137</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add routing to the app
</commit_message>
<xml_diff>
--- a/ticket-tracker.xlsx
+++ b/ticket-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhatt\projects\codex\between-the-lines\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C7DF996-7B68-4E42-A32E-FFDD1931DB7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB2B4AAA-933F-43F1-908B-BA748744D428}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
   <si>
     <t>Project Ticket Tracker</t>
   </si>
@@ -136,6 +136,18 @@
   </si>
   <si>
     <t>Staging</t>
+  </si>
+  <si>
+    <t>Auth: validate stored JWT and load current user session</t>
+  </si>
+  <si>
+    <t>Create a protected endpoint and enable authenticated users access it</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>27/04/2026</t>
   </si>
 </sst>
 </file>
@@ -549,7 +561,7 @@
       </c>
       <c r="B3" s="1">
         <f>COUNTIF(Tickets!F2:F200,"Open")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -597,7 +609,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="15" style="5" customWidth="1"/>
@@ -720,6 +732,26 @@
       </c>
       <c r="H4" s="7">
         <v>46137</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="C5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -756,5 +788,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>